<commit_message>
📊 Actualizar PROYECCION_VENTAS_DIA_PF.xlsx — 08-04-2026, 12:07:59 p. m.
</commit_message>
<xml_diff>
--- a/datos/PROYECCION_VENTAS_DIA_PF.xlsx
+++ b/datos/PROYECCION_VENTAS_DIA_PF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df502c28020c5b60/Documentos/GIM/Proteccion Familiar/Estrategia/Estrategia 2026/3.Estrategia Comercial 2026/Dash board/Archivos_Base Marzo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/ABRIL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{97D33487-474D-4B51-BD20-79F53FDD45AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37FEF0AF-1F4F-4B00-8232-71338D0CC9CF}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{B0D40A13-F561-4D6A-B9A0-4DDA76574C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0A36B42-D081-4CFE-BF28-F3D176D06970}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{97D2A031-07BF-4B71-BC0E-1411959519BA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{97D2A031-07BF-4B71-BC0E-1411959519BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyeccion Venta Diaria Q" sheetId="2" r:id="rId1"/>
@@ -68,7 +68,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -123,7 +123,7 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -134,7 +134,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares [0]" xfId="2" builtinId="6"/>
@@ -497,23 +497,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6921A9B2-21D4-4B0E-BEC1-20DEACA014A6}">
   <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.46484375" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="4">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -530,16 +530,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>3.6956290771551811E-2</v>
+        <v>2.5350997619452881E-2</v>
       </c>
       <c r="C3" s="4">
         <f>+$B$1*B3</f>
-        <v>4.2130171479569061</v>
+        <v>3.853351638156838</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -547,471 +547,471 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>7.0730541212468925E-2</v>
+        <v>5.2547401190426904E-2</v>
       </c>
       <c r="C4" s="4">
         <f t="shared" ref="C4:C33" si="0">+$B$1*B4</f>
-        <v>8.0632816982214575</v>
+        <v>7.9872049809448891</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" ref="E4:E33" si="1">+($B$1*(D4*$B$33)/C4)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>0.10384163815335309</v>
+        <v>7.7694014952965212E-2</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="0"/>
-        <v>11.837946749482253</v>
+        <v>11.809490272850713</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>0.13186797473732448</v>
+        <v>9.858003547862787E-2</v>
       </c>
       <c r="C6" s="4">
         <f t="shared" si="0"/>
-        <v>15.03294912005499</v>
+        <v>14.984165392751436</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>0.15931174916905069</v>
+        <v>0.11917477492816796</v>
       </c>
       <c r="C7" s="4">
         <f t="shared" si="0"/>
-        <v>18.161539405271778</v>
+        <v>18.114565789081528</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>0.17339439912854135</v>
+        <v>0.15714393495945966</v>
       </c>
       <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>19.766961500653714</v>
+        <v>23.885878113837869</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9" s="3">
-        <v>0.19953407243133525</v>
+        <v>0.18567768913662983</v>
       </c>
       <c r="C9" s="4">
         <f t="shared" si="0"/>
-        <v>22.746884257172219</v>
+        <v>28.223008748767732</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
       <c r="B10" s="3">
-        <v>0.21212741552113223</v>
+        <v>0.20572006514888228</v>
       </c>
       <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>24.182525369409074</v>
+        <v>31.269449902630107</v>
       </c>
       <c r="E10" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
       <c r="B11" s="3">
-        <v>0.25241833902718575</v>
+        <v>0.24992050971977844</v>
       </c>
       <c r="C11" s="4">
         <f t="shared" si="0"/>
-        <v>28.775690649099175</v>
+        <v>37.98791747740632</v>
       </c>
       <c r="E11" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
       <c r="B12" s="3">
-        <v>0.28858519729806292</v>
+        <v>0.28174964332257102</v>
       </c>
       <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>32.898712491979175</v>
+        <v>42.825945785030797</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
       <c r="B13" s="3">
-        <v>0.31916094065827749</v>
+        <v>0.31250143252845147</v>
       </c>
       <c r="C13" s="4">
         <f t="shared" si="0"/>
-        <v>36.384347235043634</v>
+        <v>47.500217744324623</v>
       </c>
       <c r="E13" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
       <c r="B14" s="3">
-        <v>0.3710932431673552</v>
+        <v>0.3539315013087635</v>
       </c>
       <c r="C14" s="4">
         <f t="shared" si="0"/>
-        <v>42.304629721078491</v>
+        <v>53.797588198932054</v>
       </c>
       <c r="E14" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
       <c r="B15" s="3">
-        <v>0.39655650496602957</v>
+        <v>0.38040883667545466</v>
       </c>
       <c r="C15" s="4">
         <f t="shared" si="0"/>
-        <v>45.207441566127372</v>
+        <v>57.822143174669108</v>
       </c>
       <c r="E15" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
       <c r="B16" s="3">
-        <v>0.41330376661630752</v>
+        <v>0.4025281719679476</v>
       </c>
       <c r="C16" s="4">
         <f t="shared" si="0"/>
-        <v>47.116629394259057</v>
+        <v>61.184282139128037</v>
       </c>
       <c r="E16" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>15</v>
       </c>
       <c r="B17" s="3">
-        <v>0.44666423331010763</v>
+        <v>0.43295410978220161</v>
       </c>
       <c r="C17" s="4">
         <f t="shared" si="0"/>
-        <v>50.919722597352269</v>
+        <v>65.809024686894645</v>
       </c>
       <c r="E17" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>0.46168480944179474</v>
+        <v>0.45249188925697992</v>
       </c>
       <c r="C18" s="4">
         <f t="shared" si="0"/>
-        <v>52.632068276364599</v>
+        <v>68.778767167060948</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>17</v>
       </c>
       <c r="B19" s="3">
-        <v>0.50976876296310047</v>
+        <v>0.50402527495234062</v>
       </c>
       <c r="C19" s="4">
         <f t="shared" si="0"/>
-        <v>58.113638977793457</v>
+        <v>76.611841792755769</v>
       </c>
       <c r="E19" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>18</v>
       </c>
       <c r="B20" s="3">
-        <v>0.53874801416457396</v>
+        <v>0.53569703113726985</v>
       </c>
       <c r="C20" s="4">
         <f t="shared" si="0"/>
-        <v>61.417273614761434</v>
+        <v>81.425948732865024</v>
       </c>
       <c r="E20" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>0.57354402285616501</v>
+        <v>0.56512252689200015</v>
       </c>
       <c r="C21" s="4">
         <f t="shared" si="0"/>
-        <v>65.384018605602819</v>
+        <v>85.898624087584025</v>
       </c>
       <c r="E21" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>0.590118708404618</v>
+        <v>0.59746485248409598</v>
       </c>
       <c r="C22" s="4">
         <f t="shared" si="0"/>
-        <v>67.27353275812645</v>
+        <v>90.814657577582594</v>
       </c>
       <c r="E22" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>0.61219544963029537</v>
+        <v>0.62740356673954634</v>
       </c>
       <c r="C23" s="4">
         <f t="shared" si="0"/>
-        <v>69.790281257853678</v>
+        <v>95.365342144411045</v>
       </c>
       <c r="E23" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>0.65080290206753511</v>
+        <v>0.65873478436710098</v>
       </c>
       <c r="C24" s="4">
         <f t="shared" si="0"/>
-        <v>74.191530835698998</v>
+        <v>100.12768722379934</v>
       </c>
       <c r="E24" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>0.67591829101271117</v>
+        <v>0.6936292485991391</v>
       </c>
       <c r="C25" s="4">
         <f t="shared" si="0"/>
-        <v>77.05468517544908</v>
+        <v>105.43164578706914</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>0.70496537561535133</v>
+        <v>0.73048956065990933</v>
       </c>
       <c r="C26" s="4">
         <f t="shared" si="0"/>
-        <v>80.366052820150045</v>
+        <v>111.03441322030622</v>
       </c>
       <c r="E26" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>25</v>
       </c>
       <c r="B27" s="3">
-        <v>0.74848013909223288</v>
+        <v>0.75740158157360793</v>
       </c>
       <c r="C27" s="4">
         <f t="shared" si="0"/>
-        <v>85.326735856514546</v>
+        <v>115.12504039918841</v>
       </c>
       <c r="E27" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>26</v>
       </c>
       <c r="B28" s="3">
-        <v>0.7883266528343289</v>
+        <v>0.79450696902884832</v>
       </c>
       <c r="C28" s="4">
         <f t="shared" si="0"/>
-        <v>89.869238423113501</v>
+        <v>120.76505929238495</v>
       </c>
       <c r="E28" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>27</v>
       </c>
       <c r="B29" s="3">
-        <v>0.80291053847691751</v>
+        <v>0.82069925549275435</v>
       </c>
       <c r="C29" s="4">
         <f t="shared" si="0"/>
-        <v>91.531801386368599</v>
+        <v>124.74628683489865</v>
       </c>
       <c r="E29" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>28</v>
       </c>
       <c r="B30" s="3">
-        <v>0.83265548488853058</v>
+        <v>0.85619028539959174</v>
       </c>
       <c r="C30" s="4">
         <f t="shared" si="0"/>
-        <v>94.922725277292486</v>
+        <v>130.14092338073795</v>
       </c>
       <c r="E30" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>29</v>
       </c>
       <c r="B31" s="3">
-        <v>0.87651827139422922</v>
+        <v>0.89014917006137573</v>
       </c>
       <c r="C31" s="4">
         <f t="shared" si="0"/>
-        <v>99.92308293894213</v>
+        <v>135.3026738493291</v>
       </c>
       <c r="E31" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>30</v>
       </c>
       <c r="B32" s="3">
-        <v>0.9449023258302931</v>
+        <v>0.94667796703885787</v>
       </c>
       <c r="C32" s="4">
         <f t="shared" si="0"/>
-        <v>107.71886514465341</v>
+        <v>143.89505098990639</v>
       </c>
       <c r="E32" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="C33" s="4">
         <f t="shared" si="0"/>
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="E33" s="4">
         <f t="shared" si="1"/>
@@ -1040,23 +1040,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFE9516D-DB2D-4859-B61B-1A68D75109AA}">
   <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.46484375" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="4">
-        <v>199791000</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+        <v>284500000</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1073,16 +1073,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>3.6956290771551811E-2</v>
+        <v>2.5350997619452881E-2</v>
       </c>
       <c r="C3" s="4">
         <f>+$B$1*B3</f>
-        <v>7383534.2895391081</v>
+        <v>7212358.8227343448</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -1090,471 +1090,471 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>7.0730541212468925E-2</v>
+        <v>5.2547401190426904E-2</v>
       </c>
       <c r="C4" s="4">
         <f t="shared" ref="C4:C33" si="0">+$B$1*B4</f>
-        <v>14131325.559380379</v>
+        <v>14949735.638676453</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" ref="E4:E33" si="1">+($B$1*(D4*$B$33)/C4)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>0.10384163815335309</v>
+        <v>7.7694014952965212E-2</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="0"/>
-        <v>20746624.728296567</v>
+        <v>22103947.254118603</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>0.13186797473732448</v>
+        <v>9.858003547862787E-2</v>
       </c>
       <c r="C6" s="4">
         <f t="shared" si="0"/>
-        <v>26346034.540744796</v>
+        <v>28046020.093669631</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>0.15931174916905069</v>
+        <v>0.11917477492816796</v>
       </c>
       <c r="C7" s="4">
         <f t="shared" si="0"/>
-        <v>31829053.678233806</v>
+        <v>33905223.467063785</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>0.17339439912854135</v>
+        <v>0.15714393495945966</v>
       </c>
       <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>34642640.396290407</v>
+        <v>44707449.495966271</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9" s="3">
-        <v>0.19953407243133525</v>
+        <v>0.18567768913662983</v>
       </c>
       <c r="C9" s="4">
         <f t="shared" si="0"/>
-        <v>39865111.865128905</v>
+        <v>52825302.559371188</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
       <c r="B10" s="3">
-        <v>0.21212741552113223</v>
+        <v>0.20572006514888228</v>
       </c>
       <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>42381148.474382527</v>
+        <v>58527358.534857005</v>
       </c>
       <c r="E10" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
       <c r="B11" s="3">
-        <v>0.25241833902718575</v>
+        <v>0.24992050971977844</v>
       </c>
       <c r="C11" s="4">
         <f t="shared" si="0"/>
-        <v>50430912.372580469</v>
+        <v>71102385.015276968</v>
       </c>
       <c r="E11" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
       <c r="B12" s="3">
-        <v>0.28858519729806292</v>
+        <v>0.28174964332257102</v>
       </c>
       <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>57656725.153377287</v>
+        <v>80157773.52527146</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
       <c r="B13" s="3">
-        <v>0.31916094065827749</v>
+        <v>0.31250143252845147</v>
       </c>
       <c r="C13" s="4">
         <f t="shared" si="0"/>
-        <v>63765483.495057918</v>
+        <v>88906657.554344445</v>
       </c>
       <c r="E13" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
       <c r="B14" s="3">
-        <v>0.3710932431673552</v>
+        <v>0.3539315013087635</v>
       </c>
       <c r="C14" s="4">
         <f t="shared" si="0"/>
-        <v>74141090.145649061</v>
+        <v>100693512.12234321</v>
       </c>
       <c r="E14" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
       <c r="B15" s="3">
-        <v>0.39655650496602957</v>
+        <v>0.38040883667545466</v>
       </c>
       <c r="C15" s="4">
         <f t="shared" si="0"/>
-        <v>79228420.683668017</v>
+        <v>108226314.03416686</v>
       </c>
       <c r="E15" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
       <c r="B16" s="3">
-        <v>0.41330376661630752</v>
+        <v>0.4025281719679476</v>
       </c>
       <c r="C16" s="4">
         <f t="shared" si="0"/>
-        <v>82574372.836038694</v>
+        <v>114519264.92488109</v>
       </c>
       <c r="E16" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>15</v>
       </c>
       <c r="B17" s="3">
-        <v>0.44666423331010763</v>
+        <v>0.43295410978220161</v>
       </c>
       <c r="C17" s="4">
         <f t="shared" si="0"/>
-        <v>89239493.83725971</v>
+        <v>123175444.23303635</v>
       </c>
       <c r="E17" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>0.46168480944179474</v>
+        <v>0.45249188925697992</v>
       </c>
       <c r="C18" s="4">
         <f t="shared" si="0"/>
-        <v>92240469.76318562</v>
+        <v>128733942.49361078</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>17</v>
       </c>
       <c r="B19" s="3">
-        <v>0.50976876296310047</v>
+        <v>0.50402527495234062</v>
       </c>
       <c r="C19" s="4">
         <f t="shared" si="0"/>
-        <v>101847210.9211608</v>
+        <v>143395190.72394091</v>
       </c>
       <c r="E19" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>18</v>
       </c>
       <c r="B20" s="3">
-        <v>0.53874801416457396</v>
+        <v>0.53569703113726985</v>
       </c>
       <c r="C20" s="4">
         <f t="shared" si="0"/>
-        <v>107637004.4979544</v>
+        <v>152405805.35855326</v>
       </c>
       <c r="E20" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>0.57354402285616501</v>
+        <v>0.56512252689200015</v>
       </c>
       <c r="C21" s="4">
         <f t="shared" si="0"/>
-        <v>114588933.87045607</v>
+        <v>160777358.90077403</v>
       </c>
       <c r="E21" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>0.590118708404618</v>
+        <v>0.59746485248409598</v>
       </c>
       <c r="C22" s="4">
         <f t="shared" si="0"/>
-        <v>117900406.87086703</v>
+        <v>169978750.53172532</v>
       </c>
       <c r="E22" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>0.61219544963029537</v>
+        <v>0.62740356673954634</v>
       </c>
       <c r="C23" s="4">
         <f t="shared" si="0"/>
-        <v>122311141.07708634</v>
+        <v>178496314.73740092</v>
       </c>
       <c r="E23" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>0.65080290206753511</v>
+        <v>0.65873478436710098</v>
       </c>
       <c r="C24" s="4">
         <f t="shared" si="0"/>
-        <v>130024562.6069749</v>
+        <v>187410046.15244022</v>
       </c>
       <c r="E24" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>0.67591829101271117</v>
+        <v>0.6936292485991391</v>
       </c>
       <c r="C25" s="4">
         <f t="shared" si="0"/>
-        <v>135042391.27972057</v>
+        <v>197337521.22645506</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>0.70496537561535133</v>
+        <v>0.73048956065990933</v>
       </c>
       <c r="C26" s="4">
         <f t="shared" si="0"/>
-        <v>140845737.35956666</v>
+        <v>207824280.00774419</v>
       </c>
       <c r="E26" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>25</v>
       </c>
       <c r="B27" s="3">
-        <v>0.74848013909223288</v>
+        <v>0.75740158157360793</v>
       </c>
       <c r="C27" s="4">
         <f t="shared" si="0"/>
-        <v>149539595.4693763</v>
+        <v>215480749.95769146</v>
       </c>
       <c r="E27" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>26</v>
       </c>
       <c r="B28" s="3">
-        <v>0.7883266528343289</v>
+        <v>0.79450696902884832</v>
       </c>
       <c r="C28" s="4">
         <f t="shared" si="0"/>
-        <v>157500570.29642341</v>
+        <v>226037232.68870735</v>
       </c>
       <c r="E28" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>27</v>
       </c>
       <c r="B29" s="3">
-        <v>0.80291053847691751</v>
+        <v>0.82069925549275435</v>
       </c>
       <c r="C29" s="4">
         <f t="shared" si="0"/>
-        <v>160414299.39284182</v>
+        <v>233488938.18768862</v>
       </c>
       <c r="E29" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>28</v>
       </c>
       <c r="B30" s="3">
-        <v>0.83265548488853058</v>
+        <v>0.85619028539959174</v>
       </c>
       <c r="C30" s="4">
         <f t="shared" si="0"/>
-        <v>166357071.9813644</v>
+        <v>243586136.19618386</v>
       </c>
       <c r="E30" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>29</v>
       </c>
       <c r="B31" s="3">
-        <v>0.87651827139422922</v>
+        <v>0.89014917006137573</v>
       </c>
       <c r="C31" s="4">
         <f t="shared" si="0"/>
-        <v>175120461.96012446</v>
+        <v>253247438.8824614</v>
       </c>
       <c r="E31" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>30</v>
       </c>
       <c r="B32" s="3">
-        <v>0.9449023258302931</v>
+        <v>0.94667796703885787</v>
       </c>
       <c r="C32" s="4">
         <f t="shared" si="0"/>
-        <v>188782980.57996008</v>
+        <v>269329881.62255508</v>
       </c>
       <c r="E32" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="C33" s="4">
         <f t="shared" si="0"/>
-        <v>199791000</v>
+        <v>284500000</v>
       </c>
       <c r="E33" s="4">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
📊 Actualizar PROYECCION_VENTAS_DIA_PF.xlsx — 14-04-2026, 2:12:43 p. m.
</commit_message>
<xml_diff>
--- a/datos/PROYECCION_VENTAS_DIA_PF.xlsx
+++ b/datos/PROYECCION_VENTAS_DIA_PF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/ABRIL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{B0D40A13-F561-4D6A-B9A0-4DDA76574C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0A36B42-D081-4CFE-BF28-F3D176D06970}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{B0D40A13-F561-4D6A-B9A0-4DDA76574C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AE06CAD-4DEF-470A-A3A5-8254FD014E3D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{97D2A031-07BF-4B71-BC0E-1411959519BA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{97D2A031-07BF-4B71-BC0E-1411959519BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyeccion Venta Diaria Q" sheetId="2" r:id="rId1"/>
@@ -125,7 +125,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -135,6 +135,7 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares [0]" xfId="2" builtinId="6"/>
@@ -177,6 +178,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1052,8 +1057,8 @@
       <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="4">
-        <v>284500000</v>
+      <c r="B1" s="5">
+        <v>321000000</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1082,7 +1087,7 @@
       </c>
       <c r="C3" s="4">
         <f>+$B$1*B3</f>
-        <v>7212358.8227343448</v>
+        <v>8137670.2358443746</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -1099,7 +1104,7 @@
       </c>
       <c r="C4" s="4">
         <f t="shared" ref="C4:C33" si="0">+$B$1*B4</f>
-        <v>14949735.638676453</v>
+        <v>16867715.782127038</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" ref="E4:E33" si="1">+($B$1*(D4*$B$33)/C4)</f>
@@ -1115,7 +1120,7 @@
       </c>
       <c r="C5" s="4">
         <f t="shared" si="0"/>
-        <v>22103947.254118603</v>
+        <v>24939778.799901832</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="1"/>
@@ -1131,7 +1136,7 @@
       </c>
       <c r="C6" s="4">
         <f t="shared" si="0"/>
-        <v>28046020.093669631</v>
+        <v>31644191.388639547</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="1"/>
@@ -1147,7 +1152,7 @@
       </c>
       <c r="C7" s="4">
         <f t="shared" si="0"/>
-        <v>33905223.467063785</v>
+        <v>38255102.751941912</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="1"/>
@@ -1163,7 +1168,7 @@
       </c>
       <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>44707449.495966271</v>
+        <v>50443203.121986553</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="1"/>
@@ -1179,7 +1184,7 @@
       </c>
       <c r="C9" s="4">
         <f t="shared" si="0"/>
-        <v>52825302.559371188</v>
+        <v>59602538.21285817</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="1"/>
@@ -1195,7 +1200,7 @@
       </c>
       <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>58527358.534857005</v>
+        <v>66036140.912791207</v>
       </c>
       <c r="E10" s="4">
         <f t="shared" si="1"/>
@@ -1211,7 +1216,7 @@
       </c>
       <c r="C11" s="4">
         <f t="shared" si="0"/>
-        <v>71102385.015276968</v>
+        <v>80224483.620048881</v>
       </c>
       <c r="E11" s="4">
         <f t="shared" si="1"/>
@@ -1227,7 +1232,7 @@
       </c>
       <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>80157773.52527146</v>
+        <v>90441635.50654529</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" si="1"/>
@@ -1243,7 +1248,7 @@
       </c>
       <c r="C13" s="4">
         <f t="shared" si="0"/>
-        <v>88906657.554344445</v>
+        <v>100312959.84163292</v>
       </c>
       <c r="E13" s="4">
         <f t="shared" si="1"/>
@@ -1259,7 +1264,7 @@
       </c>
       <c r="C14" s="4">
         <f t="shared" si="0"/>
-        <v>100693512.12234321</v>
+        <v>113612011.92011309</v>
       </c>
       <c r="E14" s="4">
         <f t="shared" si="1"/>
@@ -1275,7 +1280,7 @@
       </c>
       <c r="C15" s="4">
         <f t="shared" si="0"/>
-        <v>108226314.03416686</v>
+        <v>122111236.57282095</v>
       </c>
       <c r="E15" s="4">
         <f t="shared" si="1"/>
@@ -1291,7 +1296,7 @@
       </c>
       <c r="C16" s="4">
         <f t="shared" si="0"/>
-        <v>114519264.92488109</v>
+        <v>129211543.20171118</v>
       </c>
       <c r="E16" s="4">
         <f t="shared" si="1"/>
@@ -1307,7 +1312,7 @@
       </c>
       <c r="C17" s="4">
         <f t="shared" si="0"/>
-        <v>123175444.23303635</v>
+        <v>138978269.2400867</v>
       </c>
       <c r="E17" s="4">
         <f t="shared" si="1"/>
@@ -1323,7 +1328,7 @@
       </c>
       <c r="C18" s="4">
         <f t="shared" si="0"/>
-        <v>128733942.49361078</v>
+        <v>145249896.45149055</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="1"/>
@@ -1339,7 +1344,7 @@
       </c>
       <c r="C19" s="4">
         <f t="shared" si="0"/>
-        <v>143395190.72394091</v>
+        <v>161792113.25970134</v>
       </c>
       <c r="E19" s="4">
         <f t="shared" si="1"/>
@@ -1355,7 +1360,7 @@
       </c>
       <c r="C20" s="4">
         <f t="shared" si="0"/>
-        <v>152405805.35855326</v>
+        <v>171958746.99506363</v>
       </c>
       <c r="E20" s="4">
         <f t="shared" si="1"/>
@@ -1371,7 +1376,7 @@
       </c>
       <c r="C21" s="4">
         <f t="shared" si="0"/>
-        <v>160777358.90077403</v>
+        <v>181404331.13233206</v>
       </c>
       <c r="E21" s="4">
         <f t="shared" si="1"/>
@@ -1387,7 +1392,7 @@
       </c>
       <c r="C22" s="4">
         <f t="shared" si="0"/>
-        <v>169978750.53172532</v>
+        <v>191786217.64739481</v>
       </c>
       <c r="E22" s="4">
         <f t="shared" si="1"/>
@@ -1403,7 +1408,7 @@
       </c>
       <c r="C23" s="4">
         <f t="shared" si="0"/>
-        <v>178496314.73740092</v>
+        <v>201396544.92339438</v>
       </c>
       <c r="E23" s="4">
         <f t="shared" si="1"/>
@@ -1419,7 +1424,7 @@
       </c>
       <c r="C24" s="4">
         <f t="shared" si="0"/>
-        <v>187410046.15244022</v>
+        <v>211453865.7818394</v>
       </c>
       <c r="E24" s="4">
         <f t="shared" si="1"/>
@@ -1435,7 +1440,7 @@
       </c>
       <c r="C25" s="4">
         <f t="shared" si="0"/>
-        <v>197337521.22645506</v>
+        <v>222654988.80032367</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="1"/>
@@ -1451,7 +1456,7 @@
       </c>
       <c r="C26" s="4">
         <f t="shared" si="0"/>
-        <v>207824280.00774419</v>
+        <v>234487148.9718309</v>
       </c>
       <c r="E26" s="4">
         <f t="shared" si="1"/>
@@ -1467,7 +1472,7 @@
       </c>
       <c r="C27" s="4">
         <f t="shared" si="0"/>
-        <v>215480749.95769146</v>
+        <v>243125907.68512815</v>
       </c>
       <c r="E27" s="4">
         <f t="shared" si="1"/>
@@ -1483,7 +1488,7 @@
       </c>
       <c r="C28" s="4">
         <f t="shared" si="0"/>
-        <v>226037232.68870735</v>
+        <v>255036737.05826032</v>
       </c>
       <c r="E28" s="4">
         <f t="shared" si="1"/>
@@ -1499,7 +1504,7 @@
       </c>
       <c r="C29" s="4">
         <f t="shared" si="0"/>
-        <v>233488938.18768862</v>
+        <v>263444461.01317415</v>
       </c>
       <c r="E29" s="4">
         <f t="shared" si="1"/>
@@ -1515,7 +1520,7 @@
       </c>
       <c r="C30" s="4">
         <f t="shared" si="0"/>
-        <v>243586136.19618386</v>
+        <v>274837081.61326897</v>
       </c>
       <c r="E30" s="4">
         <f t="shared" si="1"/>
@@ -1531,7 +1536,7 @@
       </c>
       <c r="C31" s="4">
         <f t="shared" si="0"/>
-        <v>253247438.8824614</v>
+        <v>285737883.58970159</v>
       </c>
       <c r="E31" s="4">
         <f t="shared" si="1"/>
@@ -1547,7 +1552,7 @@
       </c>
       <c r="C32" s="4">
         <f t="shared" si="0"/>
-        <v>269329881.62255508</v>
+        <v>303883627.41947335</v>
       </c>
       <c r="E32" s="4">
         <f t="shared" si="1"/>
@@ -1563,7 +1568,7 @@
       </c>
       <c r="C33" s="4">
         <f t="shared" si="0"/>
-        <v>284500000</v>
+        <v>321000000</v>
       </c>
       <c r="E33" s="4">
         <f t="shared" si="1"/>

</xml_diff>